<commit_message>
fixed data validation error in xslope_earth_dam_down.xlsx
</commit_message>
<xml_diff>
--- a/docs/unit2/07_seep_slope/files/xslope_earth_dam_down.xlsx
+++ b/docs/unit2/07_seep_slope/files/xslope_earth_dam_down.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/ce544/docs/unit2/07_seep_slope/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1F3AA4-20C3-0240-A37A-1738C405BE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFCEFDE-A4A1-4A42-8B5A-E322DF8C8BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27900" yWindow="3320" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="27900" yWindow="3320" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1053,19 +1053,22 @@
     <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1085,9 +1088,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8079,11 +8079,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -8602,34 +8602,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="53" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="E2" s="48" t="s">
+      <c r="C2" s="53"/>
+      <c r="E2" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="F2" s="48"/>
-      <c r="H2" s="48" t="s">
+      <c r="F2" s="49"/>
+      <c r="H2" s="49" t="s">
         <v>136</v>
       </c>
-      <c r="I2" s="48"/>
-      <c r="K2" s="48" t="s">
+      <c r="I2" s="49"/>
+      <c r="K2" s="49" t="s">
         <v>137</v>
       </c>
-      <c r="L2" s="48"/>
-      <c r="N2" s="48" t="s">
+      <c r="L2" s="49"/>
+      <c r="N2" s="49" t="s">
         <v>138</v>
       </c>
-      <c r="O2" s="48"/>
-      <c r="Q2" s="48" t="s">
+      <c r="O2" s="49"/>
+      <c r="Q2" s="49" t="s">
         <v>139</v>
       </c>
-      <c r="R2" s="48"/>
+      <c r="R2" s="49"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
       <c r="E3" s="37" t="s">
         <v>97</v>
       </c>
@@ -9022,34 +9022,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="E2" s="49" t="s">
+      <c r="C2" s="54"/>
+      <c r="E2" s="50" t="s">
         <v>141</v>
       </c>
-      <c r="F2" s="49"/>
-      <c r="H2" s="49" t="s">
+      <c r="F2" s="50"/>
+      <c r="H2" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="I2" s="49"/>
-      <c r="K2" s="49" t="s">
+      <c r="I2" s="50"/>
+      <c r="K2" s="50" t="s">
         <v>144</v>
       </c>
-      <c r="L2" s="49"/>
-      <c r="N2" s="49" t="s">
+      <c r="L2" s="50"/>
+      <c r="N2" s="50" t="s">
         <v>145</v>
       </c>
-      <c r="O2" s="49"/>
-      <c r="Q2" s="49" t="s">
+      <c r="O2" s="50"/>
+      <c r="Q2" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="R2" s="49"/>
+      <c r="R2" s="50"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
       <c r="E3" s="39" t="s">
         <v>97</v>
       </c>
@@ -9487,36 +9487,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="44"/>
-      <c r="J7" s="44"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="45"/>
+      <c r="J7" s="45"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="44" t="s">
+      <c r="L7" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="44"/>
-      <c r="N7" s="44"/>
-      <c r="O7" s="44"/>
-      <c r="P7" s="44"/>
-      <c r="Q7" s="44"/>
-      <c r="R7" s="44" t="s">
+      <c r="M7" s="45"/>
+      <c r="N7" s="45"/>
+      <c r="O7" s="45"/>
+      <c r="P7" s="45"/>
+      <c r="Q7" s="45"/>
+      <c r="R7" s="45" t="s">
         <v>95</v>
       </c>
-      <c r="S7" s="44"/>
-      <c r="T7" s="44"/>
-      <c r="U7" s="44"/>
-      <c r="V7" s="44"/>
-      <c r="W7" s="44" t="s">
+      <c r="S7" s="45"/>
+      <c r="T7" s="45"/>
+      <c r="U7" s="45"/>
+      <c r="V7" s="45"/>
+      <c r="W7" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="X7" s="44"/>
+      <c r="X7" s="45"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -9629,7 +9629,7 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
-      <c r="W9" s="54">
+      <c r="W9" s="43">
         <v>700000</v>
       </c>
       <c r="X9" s="17">
@@ -9677,7 +9677,7 @@
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
-      <c r="W10" s="54">
+      <c r="W10" s="43">
         <v>700000</v>
       </c>
       <c r="X10" s="17">
@@ -9725,7 +9725,7 @@
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
-      <c r="W11" s="54">
+      <c r="W11" s="43">
         <v>700000</v>
       </c>
       <c r="X11" s="17">
@@ -9769,7 +9769,7 @@
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
-      <c r="W12" s="54">
+      <c r="W12" s="43">
         <v>700000</v>
       </c>
       <c r="X12" s="17">
@@ -10396,15 +10396,12 @@
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D13:D50" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
       <formula1>$C$3:$C$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K13:K50" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K9:K50" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
       <formula1>$J$3:$J$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K9:K12" xr:uid="{F449EC88-55D7-AF46-91D9-502B4AAE8A8B}">
-      <formula1>$C$26:$C$28</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9:D12" xr:uid="{F6CF285D-AF8C-554B-AF85-6DFB49CE3E59}">
       <formula1>$C$22:$C$23</formula1>
@@ -10452,74 +10449,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="D4" s="45" t="s">
+      <c r="B4" s="48"/>
+      <c r="D4" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="G4" s="45" t="s">
+      <c r="E4" s="48"/>
+      <c r="G4" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="45"/>
-      <c r="J4" s="45" t="s">
+      <c r="H4" s="48"/>
+      <c r="J4" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="M4" s="45" t="s">
+      <c r="K4" s="48"/>
+      <c r="M4" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="45"/>
-      <c r="P4" s="45" t="s">
+      <c r="N4" s="48"/>
+      <c r="P4" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="45"/>
+      <c r="Q4" s="48"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="45"/>
+      <c r="T4" s="48"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="45"/>
+      <c r="W4" s="48"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="45" t="s">
+      <c r="Y4" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="45"/>
+      <c r="Z4" s="48"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="45" t="s">
+      <c r="AB4" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="45"/>
-      <c r="AE4" s="45" t="s">
+      <c r="AC4" s="48"/>
+      <c r="AE4" s="48" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="45"/>
+      <c r="AF4" s="48"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="45" t="s">
+      <c r="AH4" s="48" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="45"/>
+      <c r="AI4" s="48"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="45" t="s">
+      <c r="AK4" s="48" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="45"/>
+      <c r="AL4" s="48"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="45" t="s">
+      <c r="AN4" s="48" t="s">
         <v>119</v>
       </c>
-      <c r="AO4" s="45"/>
+      <c r="AO4" s="48"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="45" t="s">
+      <c r="AQ4" s="48" t="s">
         <v>120</v>
       </c>
-      <c r="AR4" s="45"/>
+      <c r="AR4" s="48"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -11656,36 +11653,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11701,14 +11698,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="D2" s="49" t="s">
+      <c r="B2" s="49"/>
+      <c r="D2" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="49"/>
+      <c r="E2" s="50"/>
       <c r="G2" s="24" t="s">
         <v>85</v>
       </c>
@@ -12287,36 +12284,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="51" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="F2" s="50" t="s">
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="F2" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="J2" s="50" t="s">
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="J2" s="51" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
-      <c r="N2" s="50" t="s">
+      <c r="K2" s="51"/>
+      <c r="L2" s="51"/>
+      <c r="N2" s="51" t="s">
         <v>132</v>
       </c>
-      <c r="O2" s="50"/>
-      <c r="P2" s="50"/>
-      <c r="R2" s="50" t="s">
+      <c r="O2" s="51"/>
+      <c r="P2" s="51"/>
+      <c r="R2" s="51" t="s">
         <v>133</v>
       </c>
-      <c r="S2" s="50"/>
-      <c r="T2" s="50"/>
-      <c r="V2" s="50" t="s">
+      <c r="S2" s="51"/>
+      <c r="T2" s="51"/>
+      <c r="V2" s="51" t="s">
         <v>134</v>
       </c>
-      <c r="W2" s="50"/>
-      <c r="X2" s="50"/>
+      <c r="W2" s="51"/>
+      <c r="X2" s="51"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -12805,36 +12802,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="52" t="s">
         <v>147</v>
       </c>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="F2" s="51" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="F2" s="52" t="s">
         <v>148</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="J2" s="51" t="s">
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="J2" s="52" t="s">
         <v>149</v>
       </c>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="N2" s="51" t="s">
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="N2" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
-      <c r="R2" s="51" t="s">
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="R2" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="S2" s="51"/>
-      <c r="T2" s="51"/>
-      <c r="V2" s="51" t="s">
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="V2" s="52" t="s">
         <v>152</v>
       </c>
-      <c r="W2" s="51"/>
-      <c r="X2" s="51"/>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
fixed wrong max depth for earth dam problems
</commit_message>
<xml_diff>
--- a/docs/unit2/07_seep_slope/files/xslope_earth_dam_down.xlsx
+++ b/docs/unit2/07_seep_slope/files/xslope_earth_dam_down.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/ce544/docs/unit2/07_seep_slope/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFCEFDE-A4A1-4A42-8B5A-E322DF8C8BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD344352-2E70-CC4C-A069-955A3C3B44DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27900" yWindow="3320" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="27900" yWindow="3320" windowWidth="34200" windowHeight="20240" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1062,13 +1062,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -10442,81 +10442,81 @@
         <v>46</v>
       </c>
       <c r="B2" s="3">
-        <v>120</v>
+        <v>182</v>
       </c>
       <c r="D2" s="27" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="46"/>
+      <c r="D4" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="G4" s="48" t="s">
+      <c r="E4" s="46"/>
+      <c r="G4" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="J4" s="48" t="s">
+      <c r="H4" s="46"/>
+      <c r="J4" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="48"/>
-      <c r="M4" s="48" t="s">
+      <c r="K4" s="46"/>
+      <c r="M4" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="P4" s="48" t="s">
+      <c r="N4" s="46"/>
+      <c r="P4" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="48"/>
+      <c r="Q4" s="46"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="48" t="s">
+      <c r="S4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="48"/>
+      <c r="T4" s="46"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="48" t="s">
+      <c r="V4" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="48"/>
+      <c r="W4" s="46"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="48" t="s">
+      <c r="Y4" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="48"/>
+      <c r="Z4" s="46"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="48" t="s">
+      <c r="AB4" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="48"/>
-      <c r="AE4" s="48" t="s">
+      <c r="AC4" s="46"/>
+      <c r="AE4" s="46" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="48"/>
+      <c r="AF4" s="46"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="48" t="s">
+      <c r="AH4" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="48"/>
+      <c r="AI4" s="46"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="48" t="s">
+      <c r="AK4" s="46" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="48"/>
+      <c r="AL4" s="46"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="48" t="s">
+      <c r="AN4" s="46" t="s">
         <v>119</v>
       </c>
-      <c r="AO4" s="48"/>
+      <c r="AO4" s="46"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="48" t="s">
+      <c r="AQ4" s="46" t="s">
         <v>120</v>
       </c>
-      <c r="AR4" s="48"/>
+      <c r="AR4" s="46"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -10619,89 +10619,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="47" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Shell</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="48"/>
+      <c r="D6" s="47" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Core</v>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="48"/>
+      <c r="G6" s="47" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Clay</v>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="48"/>
+      <c r="J6" s="47" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Sand</v>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="48"/>
+      <c r="M6" s="47" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="48"/>
+      <c r="P6" s="47" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="48"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="47" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="48"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="47" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="48"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="47" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="48"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="48"/>
+      <c r="AE6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="48"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="48"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="48"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="48"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="48"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11653,36 +11653,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated everything that used earth dam problem to fix max depth error
</commit_message>
<xml_diff>
--- a/docs/unit2/07_seep_slope/files/xslope_earth_dam_down.xlsx
+++ b/docs/unit2/07_seep_slope/files/xslope_earth_dam_down.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/ce544/docs/unit2/07_seep_slope/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD344352-2E70-CC4C-A069-955A3C3B44DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D5F722-2FA1-6F40-A15F-6B357C5C0B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27900" yWindow="3320" windowWidth="34200" windowHeight="20240" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="27900" yWindow="3320" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1056,19 +1056,19 @@
     <xf numFmtId="1" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -8079,11 +8079,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -9487,36 +9487,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="45" t="s">
+      <c r="L7" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
-      <c r="O7" s="45"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45" t="s">
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="48"/>
+      <c r="R7" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="S7" s="45"/>
-      <c r="T7" s="45"/>
-      <c r="U7" s="45"/>
-      <c r="V7" s="45"/>
-      <c r="W7" s="45" t="s">
+      <c r="S7" s="48"/>
+      <c r="T7" s="48"/>
+      <c r="U7" s="48"/>
+      <c r="V7" s="48"/>
+      <c r="W7" s="48" t="s">
         <v>102</v>
       </c>
-      <c r="X7" s="45"/>
+      <c r="X7" s="48"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -9629,12 +9629,8 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
-      <c r="W9" s="43">
-        <v>700000</v>
-      </c>
-      <c r="X9" s="17">
-        <v>0.3</v>
-      </c>
+      <c r="W9" s="43"/>
+      <c r="X9" s="17"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
@@ -9677,12 +9673,8 @@
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
-      <c r="W10" s="43">
-        <v>700000</v>
-      </c>
-      <c r="X10" s="17">
-        <v>0.3</v>
-      </c>
+      <c r="W10" s="43"/>
+      <c r="X10" s="17"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
@@ -9725,12 +9717,8 @@
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
-      <c r="W11" s="43">
-        <v>700000</v>
-      </c>
-      <c r="X11" s="17">
-        <v>0.3</v>
-      </c>
+      <c r="W11" s="43"/>
+      <c r="X11" s="17"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
@@ -9769,12 +9757,8 @@
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
-      <c r="W12" s="43">
-        <v>700000</v>
-      </c>
-      <c r="X12" s="17">
-        <v>0.3</v>
-      </c>
+      <c r="W12" s="43"/>
+      <c r="X12" s="17"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
@@ -10619,89 +10603,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="47" t="str">
+      <c r="A6" s="44" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Shell</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="D6" s="47" t="str">
+      <c r="B6" s="45"/>
+      <c r="D6" s="44" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Core</v>
       </c>
-      <c r="E6" s="48"/>
-      <c r="G6" s="47" t="str">
+      <c r="E6" s="45"/>
+      <c r="G6" s="44" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Clay</v>
       </c>
-      <c r="H6" s="48"/>
-      <c r="J6" s="47" t="str">
+      <c r="H6" s="45"/>
+      <c r="J6" s="44" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Sand</v>
       </c>
-      <c r="K6" s="48"/>
-      <c r="M6" s="47" t="str">
+      <c r="K6" s="45"/>
+      <c r="M6" s="44" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="48"/>
-      <c r="P6" s="47" t="str">
+      <c r="N6" s="45"/>
+      <c r="P6" s="44" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="48"/>
+      <c r="Q6" s="45"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="47" t="str">
+      <c r="S6" s="44" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="48"/>
+      <c r="T6" s="45"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="47" t="str">
+      <c r="V6" s="44" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="48"/>
+      <c r="W6" s="45"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="47" t="str">
+      <c r="Y6" s="44" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="48"/>
+      <c r="Z6" s="45"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="47" t="str">
+      <c r="AB6" s="44" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="48"/>
-      <c r="AE6" s="47" t="str">
+      <c r="AC6" s="45"/>
+      <c r="AE6" s="44" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="48"/>
+      <c r="AF6" s="45"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="47" t="str">
+      <c r="AH6" s="44" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="48"/>
+      <c r="AI6" s="45"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="47" t="str">
+      <c r="AK6" s="44" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="48"/>
+      <c r="AL6" s="45"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="47" t="str">
+      <c r="AN6" s="44" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="48"/>
+      <c r="AO6" s="45"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="47" t="str">
+      <c r="AQ6" s="44" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="48"/>
+      <c r="AR6" s="45"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11653,36 +11637,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>